<commit_message>
Update Sheet 6 (Overall RACI) and Sheet 7 (Project RACI) with Smart SCADA content
- Sheet 6: 18 rows covering Infrastructure (Server/Hosting, OPC UA Network,
  SW License, Client Devices) and Application (Smart SCADA Ph1/Ph2, OPC UA
  integration, UI/UX NAMiQ, Database) with DEV/SIT/UAT/PROD RACI assignments
- Sheet 7: 41 rows across 8 phases (Requirement, Designing, Development, SIT,
  Testing, Commissioning, HyperCare, Handover) with SCIL/CUST columns;
  ECST column cleared; activities updated for Smart SCADA (OPC UA tag list,
  React.js/.NET dev, NAMiQ wireframes, source code handover to Zeppelin)

https://claude.ai/code/session_017vscFt44axJyw8N6Z6B9Vj
</commit_message>
<xml_diff>
--- a/SCE_Zeppelin_Mixer_R1.xlsx
+++ b/SCE_Zeppelin_Mixer_R1.xlsx
@@ -53,8 +53,8 @@
     <numFmt numFmtId="167" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="&quot;₹&quot;\ #,##0"/>
-    <numFmt numFmtId="170" formatCode="_-* #,##0.00\ _D_M_-;\-* #,##0.00\ _D_M_-;_-* &quot;-&quot;??\ _D_M_-;_-@_-"/>
-    <numFmt numFmtId="171" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="170" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="171" formatCode="_-* #,##0.00\ _D_M_-;\-* #,##0.00\ _D_M_-;_-* &quot;-&quot;??\ _D_M_-;_-@_-"/>
   </numFmts>
   <fonts count="61">
     <font>
@@ -1834,12 +1834,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="15" borderId="70"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="68"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="69"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="67"/>
@@ -1861,7 +1861,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="587">
+  <cellXfs count="589">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3372,10 +3372,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="3" borderId="8" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="7" fillId="3" borderId="8" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="3" borderId="10" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="7" fillId="3" borderId="10" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3655,6 +3655,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="86" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="3" borderId="8" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="3" borderId="10" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="24">
@@ -6464,7 +6470,7 @@
         </is>
       </c>
       <c r="C13" s="477" t="n"/>
-      <c r="D13" s="478" t="n">
+      <c r="D13" s="587" t="n">
         <v>46183</v>
       </c>
     </row>
@@ -6480,7 +6486,7 @@
         </is>
       </c>
       <c r="C14" s="473" t="n"/>
-      <c r="D14" s="479" t="n">
+      <c r="D14" s="588" t="n">
         <v>46183</v>
       </c>
     </row>
@@ -10168,7 +10174,7 @@
     <col hidden="1" width="20.44140625" customWidth="1" min="15" max="15"/>
     <col hidden="1" width="17.33203125" customWidth="1" min="16" max="16"/>
     <col hidden="1" width="18.6640625" customWidth="1" min="17" max="23"/>
-    <col hidden="1" min="24" max="38"/>
+    <col hidden="1" width="13" customWidth="1" min="24" max="38"/>
     <col hidden="1" width="9.109375" customWidth="1" min="39" max="16384"/>
   </cols>
   <sheetData>
@@ -40553,7 +40559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1"/>
   <cols>
     <col width="6" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -40640,7 +40646,7 @@
       </c>
       <c r="B4" s="580" t="inlineStr">
         <is>
-          <t>Required IT Infrastructure.</t>
+          <t>Server / Cloud Hosting</t>
         </is>
       </c>
       <c r="C4" s="159" t="inlineStr">
@@ -40650,32 +40656,32 @@
       </c>
       <c r="D4" s="160" t="inlineStr">
         <is>
-          <t>IT Server and accessories.</t>
+          <t>AWS EC2 / On-premise server provisioning</t>
         </is>
       </c>
       <c r="E4" s="159" t="inlineStr">
         <is>
-          <t>SCIL</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F4" s="160" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>I</t>
         </is>
       </c>
       <c r="G4" s="160" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>I</t>
         </is>
       </c>
       <c r="H4" s="160" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="I4" s="161" t="inlineStr">
         <is>
-          <t>Specification and estimation recommendation by SCIL post FDS Sign off.</t>
+          <t>Customer to provide on-prem option if preferred</t>
         </is>
       </c>
     </row>
@@ -40689,37 +40695,36 @@
       </c>
       <c r="D5" s="162" t="inlineStr">
         <is>
-          <t>Data Center setup, VM Creation etc</t>
+          <t>Setup, configuration &amp; deployment environment</t>
         </is>
       </c>
       <c r="E5" s="163" t="inlineStr">
         <is>
-          <t>SCIL</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F5" s="162" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G5" s="162" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H5" s="162" t="inlineStr">
         <is>
-          <t>CUST</t>
-        </is>
-      </c>
-      <c r="I5" s="164" t="n"/>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I5" s="164" t="inlineStr"/>
     </row>
     <row r="6" ht="25.2" customHeight="1">
       <c r="A6" s="522" t="n"/>
       <c r="B6" s="581" t="inlineStr">
         <is>
-          <t>Required OT Infrastructure 
-and Network .</t>
+          <t>OT-IT Network / OPC UA Connectivity</t>
         </is>
       </c>
       <c r="C6" s="165" t="inlineStr">
@@ -40729,26 +40734,34 @@
       </c>
       <c r="D6" s="166" t="inlineStr">
         <is>
-          <t>Network components</t>
-        </is>
-      </c>
-      <c r="E6" s="165" t="n"/>
+          <t>Network switch, firewall, OPC UA tunnel if required</t>
+        </is>
+      </c>
+      <c r="E6" s="165" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="F6" s="166" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>I</t>
         </is>
       </c>
       <c r="G6" s="166" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>I</t>
         </is>
       </c>
       <c r="H6" s="166" t="inlineStr">
         <is>
-          <t>CUST</t>
-        </is>
-      </c>
-      <c r="I6" s="167" t="n"/>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="I6" s="167" t="inlineStr">
+        <is>
+          <t>Zeppelin to coordinate with plant IT</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="25.2" customHeight="1" thickBot="1">
       <c r="A7" s="522" t="n"/>
@@ -40760,32 +40773,40 @@
       </c>
       <c r="D7" s="168" t="inlineStr">
         <is>
-          <t>Installation and commissioning.</t>
-        </is>
-      </c>
-      <c r="E7" s="169" t="n"/>
+          <t>Network design &amp; OPC UA server configuration on PLC side</t>
+        </is>
+      </c>
+      <c r="E7" s="169" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="F7" s="168" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="G7" s="168" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H7" s="168" t="inlineStr">
         <is>
-          <t>CUST</t>
-        </is>
-      </c>
-      <c r="I7" s="170" t="n"/>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I7" s="170" t="inlineStr">
+        <is>
+          <t>PLC OPC UA server readiness is customer responsibility</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="25.2" customHeight="1">
       <c r="A8" s="522" t="n"/>
       <c r="B8" s="582" t="inlineStr">
         <is>
-          <t>Required AIDC devices.</t>
+          <t>Infrastructure Software License</t>
         </is>
       </c>
       <c r="C8" s="159" t="inlineStr">
@@ -40795,14 +40816,30 @@
       </c>
       <c r="D8" s="160" t="inlineStr">
         <is>
-          <t>Printer, Scanner, HMI etc.</t>
-        </is>
-      </c>
-      <c r="E8" s="159" t="n"/>
-      <c r="F8" s="160" t="n"/>
-      <c r="G8" s="160" t="n"/>
-      <c r="H8" s="160" t="n"/>
-      <c r="I8" s="171" t="n"/>
+          <t>OS, DB (MS SQL / PostgreSQL), web server licenses</t>
+        </is>
+      </c>
+      <c r="E8" s="159" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F8" s="160" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G8" s="160" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H8" s="160" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="I8" s="171" t="inlineStr"/>
     </row>
     <row r="9" ht="25.2" customHeight="1" thickBot="1">
       <c r="A9" s="522" t="n"/>
@@ -40814,20 +40851,36 @@
       </c>
       <c r="D9" s="162" t="inlineStr">
         <is>
-          <t>Installation and commissioning.</t>
-        </is>
-      </c>
-      <c r="E9" s="163" t="n"/>
-      <c r="F9" s="162" t="n"/>
-      <c r="G9" s="162" t="n"/>
-      <c r="H9" s="162" t="n"/>
-      <c r="I9" s="172" t="n"/>
+          <t>License procurement &amp; installation support</t>
+        </is>
+      </c>
+      <c r="E9" s="163" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F9" s="162" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G9" s="162" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H9" s="162" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I9" s="172" t="inlineStr"/>
     </row>
     <row r="10" ht="25.2" customHeight="1">
       <c r="A10" s="522" t="n"/>
       <c r="B10" s="583" t="inlineStr">
         <is>
-          <t>Infrastructure Software License</t>
+          <t>Client Devices / Panel PCs</t>
         </is>
       </c>
       <c r="C10" s="165" t="inlineStr">
@@ -40837,14 +40890,34 @@
       </c>
       <c r="D10" s="166" t="inlineStr">
         <is>
-          <t>Database, OS, Antivirus, Monitoring tool etc</t>
-        </is>
-      </c>
-      <c r="E10" s="165" t="n"/>
-      <c r="F10" s="166" t="n"/>
-      <c r="G10" s="166" t="n"/>
-      <c r="H10" s="166" t="n"/>
-      <c r="I10" s="167" t="n"/>
+          <t>Operator PCs / panel PCs at control room</t>
+        </is>
+      </c>
+      <c r="E10" s="165" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F10" s="166" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G10" s="166" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H10" s="166" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="I10" s="167" t="inlineStr">
+        <is>
+          <t>Supplied by customer / end-user</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="25.2" customHeight="1" thickBot="1">
       <c r="A11" s="523" t="n"/>
@@ -40856,14 +40929,34 @@
       </c>
       <c r="D11" s="173" t="inlineStr">
         <is>
-          <t>Installation of Database, OS, Antivirus etc</t>
-        </is>
-      </c>
-      <c r="E11" s="174" t="n"/>
-      <c r="F11" s="173" t="n"/>
-      <c r="G11" s="173" t="n"/>
-      <c r="H11" s="173" t="n"/>
-      <c r="I11" s="175" t="n"/>
+          <t>Browser configuration &amp; access setup</t>
+        </is>
+      </c>
+      <c r="E11" s="174" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F11" s="173" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G11" s="173" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H11" s="173" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I11" s="175" t="inlineStr">
+        <is>
+          <t>Web-based app – no thick client install</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="25.2" customHeight="1">
       <c r="A12" s="579" t="inlineStr">
@@ -40873,7 +40966,7 @@
       </c>
       <c r="B12" s="584" t="inlineStr">
         <is>
-          <t>Required IT Application.</t>
+          <t>Smart SCADA App – Phase 1</t>
         </is>
       </c>
       <c r="C12" s="159" t="inlineStr">
@@ -40883,35 +40976,30 @@
       </c>
       <c r="D12" s="176" t="inlineStr">
         <is>
-          <t>All Siemens Softwares.
- (EXPR,OPIN, RDNL etc)</t>
+          <t>NAMiQ Smart SCADA platform license (Ph1 scope)</t>
         </is>
       </c>
       <c r="E12" s="159" t="inlineStr">
         <is>
-          <t>SCIL</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F12" s="160" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>I</t>
         </is>
       </c>
       <c r="G12" s="160" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>I</t>
         </is>
       </c>
       <c r="H12" s="160" t="inlineStr">
         <is>
-          <t>CUST</t>
-        </is>
-      </c>
-      <c r="I12" s="161" t="inlineStr">
-        <is>
-          <t>Specification and estimation recommendation by SCIL post FDS Sign off.</t>
-        </is>
-      </c>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I12" s="161" t="inlineStr"/>
     </row>
     <row r="13" ht="25.2" customHeight="1" thickBot="1">
       <c r="A13" s="522" t="n"/>
@@ -40922,30 +41010,30 @@
       </c>
       <c r="D13" s="441" t="inlineStr">
         <is>
-          <t>All Siemens Softwares installation.</t>
+          <t>React.js frontend, .NET backend, OPC UA integration, User Mgmt, Licensing, DE/EN language</t>
         </is>
       </c>
       <c r="E13" s="163" t="inlineStr">
         <is>
-          <t>SCIL</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F13" s="162" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G13" s="162" t="inlineStr">
         <is>
-          <t>CUST</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H13" s="162" t="inlineStr">
         <is>
-          <t>CUST</t>
-        </is>
-      </c>
-      <c r="I13" s="164" t="n"/>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I13" s="164" t="inlineStr"/>
     </row>
     <row r="14" ht="25.2" customHeight="1">
       <c r="A14" s="522" t="n"/>
@@ -40956,15 +41044,34 @@
       </c>
       <c r="D14" s="176" t="inlineStr">
         <is>
-          <t>All Non Siemens Softwares.
- (Power BI, Tableau, etc)</t>
-        </is>
-      </c>
-      <c r="E14" s="178" t="n"/>
-      <c r="F14" s="176" t="n"/>
-      <c r="G14" s="176" t="n"/>
-      <c r="H14" s="176" t="n"/>
-      <c r="I14" s="161" t="n"/>
+          <t>OPC UA tag list provided by Zeppelin/customer</t>
+        </is>
+      </c>
+      <c r="E14" s="178" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F14" s="176" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G14" s="176" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H14" s="176" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I14" s="161" t="inlineStr">
+        <is>
+          <t>Tag list to be provided before development</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="25.2" customHeight="1" thickBot="1">
       <c r="A15" s="522" t="n"/>
@@ -40976,20 +41083,36 @@
       </c>
       <c r="D15" s="441" t="inlineStr">
         <is>
-          <t>All Non Siemens Softwares installation.</t>
-        </is>
-      </c>
-      <c r="E15" s="163" t="n"/>
-      <c r="F15" s="162" t="n"/>
-      <c r="G15" s="162" t="n"/>
-      <c r="H15" s="162" t="n"/>
-      <c r="I15" s="172" t="n"/>
+          <t>OPC UA data logger (1 s / 0.1 s), process variable mapping</t>
+        </is>
+      </c>
+      <c r="E15" s="163" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F15" s="162" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G15" s="162" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H15" s="162" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I15" s="172" t="inlineStr"/>
     </row>
     <row r="16" ht="25.2" customHeight="1">
       <c r="A16" s="522" t="n"/>
       <c r="B16" s="585" t="inlineStr">
         <is>
-          <t>Required OT Application.</t>
+          <t>UI/UX Design – NAMiQ</t>
         </is>
       </c>
       <c r="C16" s="165" t="inlineStr">
@@ -40999,15 +41122,30 @@
       </c>
       <c r="D16" s="179" t="inlineStr">
         <is>
-          <t>All Siemens Automations.
- (WinCC, PLC, etc)</t>
-        </is>
-      </c>
-      <c r="E16" s="165" t="n"/>
-      <c r="F16" s="166" t="n"/>
-      <c r="G16" s="166" t="n"/>
-      <c r="H16" s="166" t="n"/>
-      <c r="I16" s="180" t="n"/>
+          <t>Wireframes &amp; screen designs by Ricardo Klement (ZSD)</t>
+        </is>
+      </c>
+      <c r="E16" s="165" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F16" s="166" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G16" s="166" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H16" s="166" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I16" s="180" t="inlineStr"/>
     </row>
     <row r="17" ht="25.2" customHeight="1" thickBot="1">
       <c r="A17" s="522" t="n"/>
@@ -41018,14 +41156,30 @@
       </c>
       <c r="D17" s="444" t="inlineStr">
         <is>
-          <t>All Siemens Automations installation.</t>
-        </is>
-      </c>
-      <c r="E17" s="182" t="n"/>
-      <c r="F17" s="444" t="n"/>
-      <c r="G17" s="444" t="n"/>
-      <c r="H17" s="444" t="n"/>
-      <c r="I17" s="170" t="n"/>
+          <t>UI implementation in React.js per approved wireframes</t>
+        </is>
+      </c>
+      <c r="E17" s="182" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F17" s="444" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G17" s="444" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H17" s="444" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I17" s="170" t="inlineStr"/>
     </row>
     <row r="18" ht="25.2" customHeight="1">
       <c r="A18" s="522" t="n"/>
@@ -41036,15 +41190,30 @@
       </c>
       <c r="D18" s="179" t="inlineStr">
         <is>
-          <t>All Non Siemens Automations.
- (OSI PI , Kepware etc)</t>
-        </is>
-      </c>
-      <c r="E18" s="165" t="n"/>
-      <c r="F18" s="166" t="n"/>
-      <c r="G18" s="166" t="n"/>
-      <c r="H18" s="166" t="n"/>
-      <c r="I18" s="180" t="n"/>
+          <t>DB license (if MS SQL)</t>
+        </is>
+      </c>
+      <c r="E18" s="165" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F18" s="166" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G18" s="166" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H18" s="166" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="I18" s="180" t="inlineStr"/>
     </row>
     <row r="19" ht="25.2" customHeight="1" thickBot="1">
       <c r="A19" s="522" t="n"/>
@@ -41056,20 +41225,36 @@
       </c>
       <c r="D19" s="444" t="inlineStr">
         <is>
-          <t>All Non Siemens Automations installation.</t>
-        </is>
-      </c>
-      <c r="E19" s="169" t="n"/>
-      <c r="F19" s="168" t="n"/>
-      <c r="G19" s="168" t="n"/>
-      <c r="H19" s="168" t="n"/>
-      <c r="I19" s="183" t="n"/>
+          <t>Schema design, data model, retention configuration</t>
+        </is>
+      </c>
+      <c r="E19" s="169" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F19" s="168" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G19" s="168" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H19" s="168" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I19" s="183" t="inlineStr"/>
     </row>
     <row r="20" ht="25.2" customHeight="1">
       <c r="A20" s="522" t="n"/>
       <c r="B20" s="586" t="inlineStr">
         <is>
-          <t>Other dependant Applications.</t>
+          <t>Smart SCADA App – Phase 2</t>
         </is>
       </c>
       <c r="C20" s="159" t="inlineStr">
@@ -41079,15 +41264,34 @@
       </c>
       <c r="D20" s="176" t="inlineStr">
         <is>
-          <t>IT Applications to be interfaced.
-(ERP, PLM, ASRS, WMS etc )</t>
-        </is>
-      </c>
-      <c r="E20" s="159" t="n"/>
-      <c r="F20" s="160" t="n"/>
-      <c r="G20" s="160" t="n"/>
-      <c r="H20" s="160" t="n"/>
-      <c r="I20" s="171" t="n"/>
+          <t>NAMiQ Smart SCADA platform license (Ph2 scope)</t>
+        </is>
+      </c>
+      <c r="E20" s="159" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F20" s="160" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G20" s="160" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H20" s="160" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I20" s="171" t="inlineStr">
+        <is>
+          <t>Recipe, Production Order, Batch Report</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="25.2" customHeight="1" thickBot="1">
       <c r="A21" s="522" t="n"/>
@@ -41098,28 +41302,39 @@
       </c>
       <c r="D21" s="441" t="inlineStr">
         <is>
-          <t>Interface development and readiness.</t>
-        </is>
-      </c>
-      <c r="E21" s="163" t="n"/>
-      <c r="F21" s="162" t="n"/>
-      <c r="G21" s="162" t="n"/>
-      <c r="H21" s="162" t="n"/>
-      <c r="I21" s="172" t="n"/>
+          <t>Recipe Mgmt, Production Order, PLC transfer, Batch Report development</t>
+        </is>
+      </c>
+      <c r="E21" s="163" t="inlineStr">
+        <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F21" s="162" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G21" s="162" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H21" s="162" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I21" s="172" t="inlineStr">
+        <is>
+          <t>Scope subject to Ph2 sign-off</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="25.2" customHeight="1">
       <c r="A22" s="522" t="n"/>
-      <c r="C22" s="159" t="inlineStr">
-        <is>
-          <t>Supply</t>
-        </is>
-      </c>
-      <c r="D22" s="176" t="inlineStr">
-        <is>
-          <t>OT Applications to be interfaced.
-(PLC, HMI, AGV etc )</t>
-        </is>
-      </c>
+      <c r="C22" s="159" t="n"/>
+      <c r="D22" s="176" t="n"/>
       <c r="E22" s="159" t="n"/>
       <c r="F22" s="160" t="n"/>
       <c r="G22" s="160" t="n"/>
@@ -41129,16 +41344,8 @@
     <row r="23" ht="25.2" customHeight="1" thickBot="1">
       <c r="A23" s="523" t="n"/>
       <c r="B23" s="461" t="n"/>
-      <c r="C23" s="185" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="D23" s="447" t="inlineStr">
-        <is>
-          <t>Interface development and readiness.</t>
-        </is>
-      </c>
+      <c r="C23" s="185" t="n"/>
+      <c r="D23" s="447" t="n"/>
       <c r="E23" s="185" t="n"/>
       <c r="F23" s="186" t="n"/>
       <c r="G23" s="186" t="n"/>
@@ -41167,6 +41374,30 @@
       <c r="H25" s="162" t="n"/>
       <c r="I25" s="1" t="n"/>
     </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="A4:A11"/>
@@ -41274,29 +41505,25 @@
       </c>
       <c r="C3" s="268" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Project Management</t>
         </is>
       </c>
       <c r="D3" s="268" t="inlineStr">
         <is>
-          <t>Requirement gathering workshops arrangement with all Stakeholders.</t>
+          <t>Kick-off meeting &amp; project charter sign-off</t>
         </is>
       </c>
       <c r="E3" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F3" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G3" s="269" t="inlineStr">
-        <is>
           <t>C</t>
         </is>
       </c>
+      <c r="G3" s="269" t="n"/>
       <c r="H3" s="270" t="n"/>
     </row>
     <row r="4" customFormat="1" s="1">
@@ -41310,17 +41537,17 @@
       </c>
       <c r="C4" s="268" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D4" s="268" t="inlineStr">
         <is>
-          <t>Business Requirement Document creation.</t>
+          <t>Requirement review &amp; gap analysis</t>
         </is>
       </c>
       <c r="E4" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F4" s="269" t="inlineStr">
@@ -41328,11 +41555,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G4" s="269" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="G4" s="269" t="n"/>
       <c r="H4" s="270" t="n"/>
     </row>
     <row r="5" customFormat="1" s="1">
@@ -41346,29 +41569,25 @@
       </c>
       <c r="C5" s="268" t="inlineStr">
         <is>
-          <t>Requirement Checkpoint.</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D5" s="268" t="inlineStr">
         <is>
-          <t>Business Requirement Document Sign Off</t>
+          <t>OPC UA tag list provision by customer</t>
         </is>
       </c>
       <c r="E5" s="269" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>I</t>
         </is>
       </c>
       <c r="F5" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G5" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G5" s="269" t="n"/>
       <c r="H5" s="270" t="n"/>
     </row>
     <row r="6" customFormat="1" s="1">
@@ -41382,29 +41601,25 @@
       </c>
       <c r="C6" s="268" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D6" s="268" t="inlineStr">
         <is>
-          <t>User Acceptance Criteria creation</t>
+          <t>IT/OT network topology review</t>
         </is>
       </c>
       <c r="E6" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F6" s="269" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G6" s="269" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G6" s="269" t="n"/>
       <c r="H6" s="270" t="n"/>
     </row>
     <row r="7" customFormat="1" s="1">
@@ -41413,34 +41628,30 @@
       </c>
       <c r="B7" s="268" t="inlineStr">
         <is>
-          <t>Designing</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="C7" s="268" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Project Management</t>
         </is>
       </c>
       <c r="D7" s="268" t="inlineStr">
         <is>
-          <t>Conference room pilot with process owners/ business heads on need basis.</t>
+          <t>Requirement sign-off &amp; baseline freeze</t>
         </is>
       </c>
       <c r="E7" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F7" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G7" s="269" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G7" s="269" t="n"/>
       <c r="H7" s="270" t="n"/>
     </row>
     <row r="8" customFormat="1" s="1">
@@ -41454,29 +41665,25 @@
       </c>
       <c r="C8" s="268" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D8" s="268" t="inlineStr">
         <is>
-          <t>Data requirements and availibility of all application and interfaces</t>
+          <t>System architecture design (React.js / .NET / DB)</t>
         </is>
       </c>
       <c r="E8" s="269" t="inlineStr">
         <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F8" s="269" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F8" s="269" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G8" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G8" s="269" t="n"/>
       <c r="H8" s="270" t="n"/>
     </row>
     <row r="9" customFormat="1" s="1">
@@ -41490,29 +41697,25 @@
       </c>
       <c r="C9" s="268" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D9" s="268" t="inlineStr">
         <is>
-          <t>Server sizing &amp; specification recommendation.</t>
+          <t>OPC UA data model &amp; tag mapping design</t>
         </is>
       </c>
       <c r="E9" s="269" t="inlineStr">
         <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F9" s="269" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F9" s="269" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G9" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G9" s="269" t="n"/>
       <c r="H9" s="270" t="n"/>
     </row>
     <row r="10" customFormat="1" s="1">
@@ -41526,29 +41729,25 @@
       </c>
       <c r="C10" s="268" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D10" s="268" t="inlineStr">
         <is>
-          <t>AIDC ( Scarnner,printer,PDA etc ) specification recommendation .</t>
+          <t>UI/UX wireframes – NAMiQ (Ricardo Klement, ZSD)</t>
         </is>
       </c>
       <c r="E10" s="269" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F10" s="269" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G10" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G10" s="269" t="n"/>
       <c r="H10" s="270" t="n"/>
     </row>
     <row r="11" customFormat="1" s="1">
@@ -41567,24 +41766,20 @@
       </c>
       <c r="D11" s="268" t="inlineStr">
         <is>
-          <t>Overall Solution architecture document creation.</t>
+          <t>Wireframe review &amp; approval by Zeppelin</t>
         </is>
       </c>
       <c r="E11" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F11" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G11" s="269" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G11" s="269" t="n"/>
       <c r="H11" s="270" t="n"/>
     </row>
     <row r="12" customFormat="1" s="1">
@@ -41603,24 +41798,20 @@
       </c>
       <c r="D12" s="268" t="inlineStr">
         <is>
-          <t>Infrastructure architecture document creation.</t>
+          <t>Database schema design (MS SQL / PostgreSQL)</t>
         </is>
       </c>
       <c r="E12" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F12" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G12" s="269" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G12" s="269" t="n"/>
       <c r="H12" s="270" t="n"/>
     </row>
     <row r="13" customFormat="1" s="1">
@@ -41639,24 +41830,20 @@
       </c>
       <c r="D13" s="268" t="inlineStr">
         <is>
-          <t>Database requirements &amp; specifications</t>
+          <t>Data logger configuration design (1 s / 0.1 s)</t>
         </is>
       </c>
       <c r="E13" s="269" t="inlineStr">
         <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F13" s="269" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F13" s="269" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G13" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G13" s="269" t="n"/>
       <c r="H13" s="270" t="n"/>
     </row>
     <row r="14" customFormat="1" s="1">
@@ -41670,29 +41857,25 @@
       </c>
       <c r="C14" s="268" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D14" s="268" t="inlineStr">
         <is>
-          <t>Functional design documentation.</t>
+          <t>Graph &amp; process screen layout design</t>
         </is>
       </c>
       <c r="E14" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F14" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G14" s="269" t="inlineStr">
-        <is>
           <t>C</t>
         </is>
       </c>
+      <c r="G14" s="269" t="n"/>
       <c r="H14" s="270" t="n"/>
     </row>
     <row r="15" customFormat="1" s="1">
@@ -41706,29 +41889,25 @@
       </c>
       <c r="C15" s="268" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D15" s="268" t="inlineStr">
         <is>
-          <t>Interface Control design documentation</t>
+          <t>User management &amp; licensing design</t>
         </is>
       </c>
       <c r="E15" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F15" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G15" s="269" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G15" s="269" t="n"/>
       <c r="H15" s="270" t="n"/>
     </row>
     <row r="16" customFormat="1" s="1">
@@ -41742,29 +41921,25 @@
       </c>
       <c r="C16" s="268" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D16" s="268" t="inlineStr">
         <is>
-          <t>Cordination with all OEM's for disucssion and follow ICD.</t>
+          <t>Hosting &amp; deployment architecture (AWS / on-prem)</t>
         </is>
       </c>
       <c r="E16" s="269" t="inlineStr">
         <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F16" s="269" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F16" s="269" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G16" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G16" s="269" t="n"/>
       <c r="H16" s="270" t="n"/>
     </row>
     <row r="17" customFormat="1" s="1">
@@ -41778,12 +41953,12 @@
       </c>
       <c r="C17" s="268" t="inlineStr">
         <is>
-          <t>Integration Checkpoint.</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D17" s="268" t="inlineStr">
         <is>
-          <t>Interface Control design Sign Off.</t>
+          <t>Network &amp; firewall rule design for OPC UA</t>
         </is>
       </c>
       <c r="E17" s="269" t="inlineStr">
@@ -41793,14 +41968,10 @@
       </c>
       <c r="F17" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G17" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G17" s="269" t="n"/>
       <c r="H17" s="270" t="n"/>
     </row>
     <row r="18" customFormat="1" s="1">
@@ -41814,12 +41985,12 @@
       </c>
       <c r="C18" s="268" t="inlineStr">
         <is>
-          <t>Solution Checkpoint.</t>
+          <t>Project Management</t>
         </is>
       </c>
       <c r="D18" s="268" t="inlineStr">
         <is>
-          <t>Functional design Sign Off.</t>
+          <t>Design document review &amp; sign-off</t>
         </is>
       </c>
       <c r="E18" s="269" t="inlineStr">
@@ -41829,14 +42000,10 @@
       </c>
       <c r="F18" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G18" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G18" s="269" t="n"/>
       <c r="H18" s="270" t="n"/>
     </row>
     <row r="19" customFormat="1" s="1">
@@ -41845,34 +42012,30 @@
       </c>
       <c r="B19" s="268" t="inlineStr">
         <is>
-          <t>Designing</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="C19" s="268" t="inlineStr">
         <is>
-          <t>Acceptance Checkpoint.</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D19" s="268" t="inlineStr">
         <is>
-          <t>User Acceptance Criteria Sign Off.</t>
+          <t>React.js frontend development (Ph1 screens)</t>
         </is>
       </c>
       <c r="E19" s="269" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F19" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G19" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G19" s="269" t="n"/>
       <c r="H19" s="270" t="n"/>
     </row>
     <row r="20" customFormat="1" s="1">
@@ -41881,34 +42044,30 @@
       </c>
       <c r="B20" s="268" t="inlineStr">
         <is>
-          <t>Designing</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="C20" s="268" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D20" s="268" t="inlineStr">
         <is>
-          <t>Traceability matrix against Requirement IDs</t>
+          <t>.NET backend &amp; REST API development</t>
         </is>
       </c>
       <c r="E20" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F20" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G20" s="269" t="inlineStr">
-        <is>
           <t>I</t>
         </is>
       </c>
+      <c r="G20" s="269" t="n"/>
       <c r="H20" s="270" t="n"/>
     </row>
     <row r="21" customFormat="1" s="1">
@@ -41922,17 +42081,17 @@
       </c>
       <c r="C21" s="268" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D21" s="268" t="inlineStr">
         <is>
-          <t>Master and transactional data template.</t>
+          <t>OPC UA data logger module development</t>
         </is>
       </c>
       <c r="E21" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F21" s="269" t="inlineStr">
@@ -41940,11 +42099,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G21" s="269" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="G21" s="269" t="n"/>
       <c r="H21" s="270" t="n"/>
     </row>
     <row r="22" customFormat="1" s="1">
@@ -41958,29 +42113,25 @@
       </c>
       <c r="C22" s="268" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D22" s="268" t="inlineStr">
         <is>
-          <t>Master and transactional data availability in template.</t>
+          <t>User management &amp; licensing module development</t>
         </is>
       </c>
       <c r="E22" s="269" t="inlineStr">
         <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F22" s="269" t="inlineStr">
+        <is>
           <t>I</t>
         </is>
       </c>
-      <c r="F22" s="269" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G22" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G22" s="269" t="n"/>
       <c r="H22" s="270" t="n"/>
     </row>
     <row r="23" customFormat="1" s="1">
@@ -41994,29 +42145,25 @@
       </c>
       <c r="C23" s="268" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D23" s="268" t="inlineStr">
         <is>
-          <t>Master Data upload.</t>
+          <t>DE / EN language switch implementation</t>
         </is>
       </c>
       <c r="E23" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F23" s="269" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G23" s="269" t="inlineStr">
-        <is>
           <t>I</t>
         </is>
       </c>
+      <c r="G23" s="269" t="n"/>
       <c r="H23" s="270" t="n"/>
     </row>
     <row r="24" customFormat="1" s="1">
@@ -42025,22 +42172,22 @@
       </c>
       <c r="B24" s="268" t="inlineStr">
         <is>
-          <t>SIT</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="C24" s="268" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D24" s="268" t="inlineStr">
         <is>
-          <t>Readiness of all OEM's interfaces for Integration testing.</t>
+          <t>Dev/Test environment setup on server</t>
         </is>
       </c>
       <c r="E24" s="269" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F24" s="269" t="inlineStr">
@@ -42048,11 +42195,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G24" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G24" s="269" t="n"/>
       <c r="H24" s="270" t="n"/>
     </row>
     <row r="25" customFormat="1" s="1">
@@ -42061,34 +42204,30 @@
       </c>
       <c r="B25" s="268" t="inlineStr">
         <is>
-          <t>SIT</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="C25" s="268" t="inlineStr">
         <is>
-          <t>Demo</t>
+          <t>Project Management</t>
         </is>
       </c>
       <c r="D25" s="268" t="inlineStr">
         <is>
-          <t>Demo of possible feature.</t>
+          <t>Sprint reviews &amp; progress reporting</t>
         </is>
       </c>
       <c r="E25" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F25" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G25" s="269" t="inlineStr">
-        <is>
           <t>C</t>
         </is>
       </c>
+      <c r="G25" s="269" t="n"/>
       <c r="H25" s="270" t="n"/>
     </row>
     <row r="26" customFormat="1" s="1">
@@ -42102,29 +42241,25 @@
       </c>
       <c r="C26" s="268" t="inlineStr">
         <is>
-          <t>Demo</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D26" s="268" t="inlineStr">
         <is>
-          <t>Demo feedback and acceptance.</t>
+          <t>PLC OPC UA server readiness &amp; availability for SIT</t>
         </is>
       </c>
       <c r="E26" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>I</t>
         </is>
       </c>
       <c r="F26" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G26" s="269" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G26" s="269" t="n"/>
       <c r="H26" s="270" t="n"/>
     </row>
     <row r="27" customFormat="1" s="1">
@@ -42133,7 +42268,7 @@
       </c>
       <c r="B27" s="268" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>SIT</t>
         </is>
       </c>
       <c r="C27" s="268" t="inlineStr">
@@ -42143,24 +42278,20 @@
       </c>
       <c r="D27" s="268" t="inlineStr">
         <is>
-          <t>User Acceptance Criteria Testing</t>
+          <t>System integration testing – OPC UA live data</t>
         </is>
       </c>
       <c r="E27" s="269" t="inlineStr">
         <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F27" s="269" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F27" s="269" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G27" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G27" s="269" t="n"/>
       <c r="H27" s="270" t="n"/>
     </row>
     <row r="28" customFormat="1" s="1">
@@ -42169,34 +42300,30 @@
       </c>
       <c r="B28" s="268" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>SIT</t>
         </is>
       </c>
       <c r="C28" s="268" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D28" s="268" t="inlineStr">
         <is>
-          <t>UAT test plan</t>
+          <t>SIT defect resolution &amp; re-test</t>
         </is>
       </c>
       <c r="E28" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F28" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G28" s="269" t="inlineStr">
-        <is>
           <t>C</t>
         </is>
       </c>
+      <c r="G28" s="269" t="n"/>
       <c r="H28" s="270" t="n"/>
     </row>
     <row r="29" customFormat="1" s="1">
@@ -42210,12 +42337,12 @@
       </c>
       <c r="C29" s="268" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D29" s="268" t="inlineStr">
         <is>
-          <t>UAT Sign off</t>
+          <t>User acceptance testing (UAT) execution by Zeppelin</t>
         </is>
       </c>
       <c r="E29" s="269" t="inlineStr">
@@ -42225,14 +42352,10 @@
       </c>
       <c r="F29" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G29" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G29" s="269" t="n"/>
       <c r="H29" s="270" t="n"/>
     </row>
     <row r="30" customFormat="1" s="1">
@@ -42241,7 +42364,7 @@
       </c>
       <c r="B30" s="268" t="inlineStr">
         <is>
-          <t>Commissioning</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C30" s="268" t="inlineStr">
@@ -42251,24 +42374,20 @@
       </c>
       <c r="D30" s="268" t="inlineStr">
         <is>
-          <t>MES Products installation.</t>
+          <t>UAT defect logging &amp; prioritisation</t>
         </is>
       </c>
       <c r="E30" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F30" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G30" s="269" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G30" s="269" t="n"/>
       <c r="H30" s="270" t="n"/>
     </row>
     <row r="31" customFormat="1" s="1">
@@ -42277,34 +42396,30 @@
       </c>
       <c r="B31" s="268" t="inlineStr">
         <is>
-          <t>Commissioning</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C31" s="268" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D31" s="268" t="inlineStr">
         <is>
-          <t>VM, Database and other 3rd party application installation.</t>
+          <t>UAT defect fix &amp; sign-off</t>
         </is>
       </c>
       <c r="E31" s="269" t="inlineStr">
         <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F31" s="269" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F31" s="269" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G31" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G31" s="269" t="n"/>
       <c r="H31" s="270" t="n"/>
     </row>
     <row r="32" customFormat="1" s="1">
@@ -42323,24 +42438,20 @@
       </c>
       <c r="D32" s="268" t="inlineStr">
         <is>
-          <t>Server mounting,Storage configuration, OS, Antivirus, Network Readiness in Datacentre.</t>
+          <t>Production server setup &amp; deployment</t>
         </is>
       </c>
       <c r="E32" s="269" t="inlineStr">
         <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F32" s="269" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F32" s="269" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G32" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G32" s="269" t="n"/>
       <c r="H32" s="270" t="n"/>
     </row>
     <row r="33" customFormat="1" s="1">
@@ -42354,29 +42465,25 @@
       </c>
       <c r="C33" s="268" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D33" s="268" t="inlineStr">
         <is>
-          <t>Backup Software if any</t>
+          <t>Smart SCADA installation &amp; go-live configuration</t>
         </is>
       </c>
       <c r="E33" s="269" t="inlineStr">
         <is>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="F33" s="269" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F33" s="269" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G33" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G33" s="269" t="n"/>
       <c r="H33" s="270" t="n"/>
     </row>
     <row r="34" customFormat="1" s="1">
@@ -42390,17 +42497,17 @@
       </c>
       <c r="C34" s="268" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D34" s="268" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOP and user manual </t>
+          <t>OPC UA live connection validation in production</t>
         </is>
       </c>
       <c r="E34" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F34" s="269" t="inlineStr">
@@ -42408,11 +42515,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G34" s="269" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="G34" s="269" t="n"/>
       <c r="H34" s="270" t="n"/>
     </row>
     <row r="35" customFormat="1" s="1">
@@ -42426,17 +42529,17 @@
       </c>
       <c r="C35" s="268" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D35" s="268" t="inlineStr">
         <is>
-          <t>Infrastructure, Database, Backup monitoring tools installation.</t>
+          <t>Operator training – Smart SCADA usage</t>
         </is>
       </c>
       <c r="E35" s="269" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F35" s="269" t="inlineStr">
@@ -42444,11 +42547,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G35" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G35" s="269" t="n"/>
       <c r="H35" s="270" t="n"/>
     </row>
     <row r="36" ht="22.8" customFormat="1" customHeight="1" s="1">
@@ -42457,34 +42556,30 @@
       </c>
       <c r="B36" s="268" t="inlineStr">
         <is>
-          <t>HyperCare</t>
+          <t>Commissioning</t>
         </is>
       </c>
       <c r="C36" s="268" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Project Management</t>
         </is>
       </c>
       <c r="D36" s="268" t="inlineStr">
         <is>
-          <t>VM/Server Monitoring - Manually monitor the availability and performance of the Virtual Machines using OEM provided management tools at periodic intervals.</t>
+          <t>Go-live sign-off</t>
         </is>
       </c>
       <c r="E36" s="269" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F36" s="269" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G36" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G36" s="269" t="n"/>
       <c r="H36" s="270" t="n"/>
     </row>
     <row r="37" ht="22.8" customFormat="1" customHeight="1" s="1">
@@ -42503,24 +42598,20 @@
       </c>
       <c r="D37" s="268" t="inlineStr">
         <is>
-          <t>DB Monitoring - Manually monitor the availability of the databases using OEM provided management tools at periodic intervals</t>
+          <t>Post go-live monitoring &amp; issue triage</t>
         </is>
       </c>
       <c r="E37" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F37" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G37" s="269" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G37" s="269" t="n"/>
       <c r="H37" s="270" t="n"/>
     </row>
     <row r="38" customFormat="1" s="1">
@@ -42534,17 +42625,17 @@
       </c>
       <c r="C38" s="268" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D38" s="268" t="inlineStr">
         <is>
-          <t>Backup Monitoring - Monitor the failed backup jobs Backup software console at periodic intervals</t>
+          <t>Bug fixes &amp; minor enhancements (HyperCare scope)</t>
         </is>
       </c>
       <c r="E38" s="269" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F38" s="269" t="inlineStr">
@@ -42552,11 +42643,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G38" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G38" s="269" t="n"/>
       <c r="H38" s="270" t="n"/>
     </row>
     <row r="39" customFormat="1" s="1">
@@ -42570,29 +42657,25 @@
       </c>
       <c r="C39" s="268" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D39" s="268" t="inlineStr">
         <is>
-          <t>Application Monitoring : Monitor the availability of applications</t>
+          <t>Performance &amp; stability monitoring</t>
         </is>
       </c>
       <c r="E39" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F39" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G39" s="269" t="inlineStr">
-        <is>
           <t>I</t>
         </is>
       </c>
+      <c r="G39" s="269" t="n"/>
       <c r="H39" s="270" t="n"/>
     </row>
     <row r="40" ht="22.8" customFormat="1" customHeight="1" s="1">
@@ -42606,29 +42689,25 @@
       </c>
       <c r="C40" s="268" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Project Management</t>
         </is>
       </c>
       <c r="D40" s="268" t="inlineStr">
         <is>
-          <t>Performance Maintenance - configuration changes, clean-up environment, identify inefficient SQL queries, Perform scheduled database start-up/shutdown, Database recovery</t>
+          <t>HyperCare status reporting to Zeppelin</t>
         </is>
       </c>
       <c r="E40" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F40" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G40" s="269" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G40" s="269" t="n"/>
       <c r="H40" s="270" t="n"/>
     </row>
     <row r="41" ht="22.8" customFormat="1" customHeight="1" s="1">
@@ -42642,29 +42721,25 @@
       </c>
       <c r="C41" s="268" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Project Management</t>
         </is>
       </c>
       <c r="D41" s="268" t="inlineStr">
         <is>
-          <t>DB Structural Maintenance - Table space, disk space, and temporary space management, Database object structural management, Maintain physical database layout</t>
+          <t>HyperCare closure sign-off</t>
         </is>
       </c>
       <c r="E41" s="269" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F41" s="269" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G41" s="269" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="G41" s="269" t="n"/>
       <c r="H41" s="270" t="n"/>
     </row>
     <row r="42" customFormat="1" s="1">
@@ -42673,22 +42748,22 @@
       </c>
       <c r="B42" s="268" t="inlineStr">
         <is>
-          <t>HyperCare</t>
+          <t>Handover</t>
         </is>
       </c>
       <c r="C42" s="268" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D42" s="268" t="inlineStr">
         <is>
-          <t>Network Monitoring System installation</t>
+          <t>Source code &amp; documentation handover to Zeppelin</t>
         </is>
       </c>
       <c r="E42" s="269" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F42" s="269" t="inlineStr">
@@ -42696,11 +42771,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G42" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G42" s="269" t="n"/>
       <c r="H42" s="270" t="n"/>
     </row>
     <row r="43" customFormat="1" s="1">
@@ -42709,22 +42780,22 @@
       </c>
       <c r="B43" s="268" t="inlineStr">
         <is>
-          <t>HyperCare</t>
+          <t>Handover</t>
         </is>
       </c>
       <c r="C43" s="268" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Project Management</t>
         </is>
       </c>
       <c r="D43" s="268" t="inlineStr">
         <is>
-          <t>VM, Server, OS, Antivirus, other software maintenance</t>
+          <t>Final project closure &amp; lessons learned</t>
         </is>
       </c>
       <c r="E43" s="269" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F43" s="269" t="inlineStr">
@@ -42732,11 +42803,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G43" s="269" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="G43" s="269" t="n"/>
       <c r="H43" s="270" t="n"/>
     </row>
     <row r="44" customFormat="1" s="1"/>

</xml_diff>

<commit_message>
Fix Sheet 6 & 7 header rows and remove template warning text
- Sheet 6 row 1: replaced template warning with project title
- Sheet 6 row 2: added missing 'Area' column header
- Sheet 7 row 1: replaced template warning with project title
- Sheet 7 row 2: cleared ECST column header (column removed from scope)

https://claude.ai/code/session_017vscFt44axJyw8N6Z6B9Vj
</commit_message>
<xml_diff>
--- a/SCE_Zeppelin_Mixer_R1.xlsx
+++ b/SCE_Zeppelin_Mixer_R1.xlsx
@@ -40559,7 +40559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1"/>
   <cols>
     <col width="6" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -40576,12 +40576,16 @@
     <row r="1" ht="21" customHeight="1">
       <c r="A1" s="436" t="inlineStr">
         <is>
-          <t>MUST BE MODIFIED AS PER PROJECT AND INCLUDED IN TECHNICAL OFFER : Overall RACI Section</t>
+          <t>Overall RACI – Smart SCADA Mixer Data Logging &amp; Display | Zeppelin Systems GmbH, Kassel</t>
         </is>
       </c>
     </row>
     <row r="2" ht="21" customHeight="1">
-      <c r="A2" s="156" t="n"/>
+      <c r="A2" s="156" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
       <c r="B2" s="457" t="inlineStr">
         <is>
           <t>Activity</t>
@@ -41374,30 +41378,6 @@
       <c r="H25" s="162" t="n"/>
       <c r="I25" s="1" t="n"/>
     </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="A4:A11"/>
@@ -41452,7 +41432,7 @@
     <row r="1" ht="21" customHeight="1">
       <c r="A1" s="436" t="inlineStr">
         <is>
-          <t>MUST BE MODIFIED AS PER PROJECT AND INCLUDED IN TECHNICAL OFFER : Project RACI Section</t>
+          <t>Project RACI – Smart SCADA Mixer Data Logging &amp; Display | Zeppelin Systems GmbH, Kassel</t>
         </is>
       </c>
     </row>
@@ -41487,11 +41467,7 @@
           <t>CUST</t>
         </is>
       </c>
-      <c r="G2" s="149" t="inlineStr">
-        <is>
-          <t>ECST</t>
-        </is>
-      </c>
+      <c r="G2" s="149" t="n"/>
       <c r="H2" s="270" t="n"/>
     </row>
     <row r="3" customFormat="1" s="1">

</xml_diff>